<commit_message>
Add human approval workflow and .gitignore
Add new WF04_Human_Approval workflow to the project pipeline. Add .gitignore to exclude UiPath local build artifacts (.local, .project, .objects, .settings, .templates, .tmh). Update project dependencies and rebuild artifacts.
</commit_message>
<xml_diff>
--- a/Data/Trends.xlsx
+++ b/Data/Trends.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://groupecgi-my.sharepoint.com/personal/ali_mahjoub_cgi_com/Documents/Documents/UiPath/AI Social Media Manager/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{FC83683F-42BF-4097-A0B3-C26A2A443609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08CCEAE0-71E8-441E-A8C2-EC4F7C3C5AD3}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{FC83683F-42BF-4097-A0B3-C26A2A443609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28305F6E-3194-48A0-8E46-F4BBB7E0471C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{680B1045-F99F-49B7-AF7E-A924B2A05251}"/>
   </bookViews>
@@ -577,7 +577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -714,7 +714,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>30</v>
       </c>

</xml_diff>